<commit_message>
New character set. Ui fixes
</commit_message>
<xml_diff>
--- a/lores.xlsx
+++ b/lores.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\daeva\Desktop\Card_game\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22C5FAD4-F842-4B55-A44B-FAEDB9E5FFEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0656AC25-0B0B-44FB-97CD-89A35F399ACB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E9E6528D-FBE9-4018-A878-CDA73BAA7273}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="130">
   <si>
     <t>name</t>
   </si>
@@ -394,6 +394,36 @@
   </si>
   <si>
     <t>Known universally as the Calamity Demon, Samara Blackheart is an estimated four hundred and ten year old entity whose very existence is treated as a natural disaster. Fighting as a Dark attuned Soul Harvester, she brings absolute chaos and death to the battlefield with her devastating world shattering strikes. As a prominent member of the notorious half demon Blackheart family, she oversees the freezing southern expanses of the continent known as the Frozen Berg. Serving as both the head executor and chief headhunter for her cursed bloodline, her true goals and intentions during the current rise of the new demon king remain shrouded in complete mystery. Samara cemented her terrifying legacy during the second demon wars at the massacre of Sunwatch Bay, where she singlehandedly slaughtered tens of thousands of humans and entirely shattered the southern advance of the Lightspear forces. Her apocalyptic rampage was only halted when she was challenged and ultimately subjugated by a legendary coalition of heroes consisting of Reinhart Den, Odin Stormrage, and Melisande Sunward. Though she was defeated, she managed to claim the life of Melisande, the elven empress widely believed to be the reincarnate of the ancient goddess Marpha. Samara barely survived the brutal encounter and has remained entirely silent ever since, brooding in the shadows until now.</t>
+  </si>
+  <si>
+    <t>Rin Blackheart</t>
+  </si>
+  <si>
+    <t>The Obsidian Ember</t>
+  </si>
+  <si>
+    <t>Alastor Blackheart</t>
+  </si>
+  <si>
+    <t>Master of Darkness</t>
+  </si>
+  <si>
+    <t>Earth, Fire</t>
+  </si>
+  <si>
+    <t>Born at the height of the second demon wars, seventy two year old Rin is the youngest member of the notorious Blackheart family. Despite her dark lineage, she is a remarkably smart and well mannered half demon Warrior who harbors a genuine fondness for humanity. Wielding a massive obsidian blade naturally imbued with fierce Fire magic, she is a formidable melee combatant who actively fights for a peaceful coexistence rather than the destruction her kin are known for. Her goodwill was met with profound tragedy when she was hunted and captured by Serilla, the terrifying hidden weapon of the Moonlight Scripture. Enduring brutal torture and indefinite imprisonment within the citadel dungeons, her hope almost faded entirely until her former partner Morrigan Crow orchestrated her escape following a successful artifact retrieval. Now finally reunited, the two have turned their backs on the treacherous human capital, charting a perilous course deep through the dark glade toward the freezing expanse of the Frozen Berg.</t>
+  </si>
+  <si>
+    <t>Estimated to be five hundred and fifty years old, Alastor is a profoundly mysterious and expressionless Warrior who commands both Earth and Fire in a seamless blend of melee and magical combat. Whispered to be the very first half demon in existence, he made history as the original demonfolk to converse on equal grounds with the higher races in a noble bid for lasting peace. Tragically, these diplomatic efforts were shattered when the elven king fell to an unforeseeable corruption, transforming into the first demon king and immediately slaughtering Alastor's vulnerable kin. Because of his close proximity to the tragic event, many wrongfully blamed Alastor for the corruption, marking him as the primary architect behind the fall of the elven kingdom. Despite the heavy accusations, he fought alongside the ancient goddess Marpha to subjugate the mad king before vanishing entirely into the icy depths of the Frozen Berg. After his remaining kin played a major role in reclaiming the dark glade during the first demon war, this ancient pioneer has stepped out of the shadows once more, reappearing after five centuries of silence to face a world at the brink of total annihilation.</t>
+  </si>
+  <si>
+    <t>At one hundred and forty nine years old, Freya Blackheart is a Dark Berserker whose terrifying true nature earned her the moniker of The Great Cold among her fellow demonfolk. She cleverly infiltrated the ranks of the human citadel templars under a highly skittish guise, aiming to locate the living weapon Serilla and rescue a captive kin hidden deep within the dungeons. Her masterful deception held strong for a time, successfully hiding her dark origins until she was eventually cornered and exposed by the holy cleric Sylas and the ranger Kaelen. Forced to drop her timid facade, Freya revealed her true form as a vicious half demon shapeshifter hailing from the brutal Frozen Berg. Contrary to the quiet and cowardly persona she carefully crafted for the church, her actual personality is incredibly loud, mad, and unapologetically brutish. Driven by a highly cynical worldview and an insatiable bloodlust, she is a monumental threat on the battlefield, gleefully crushing anyone foolish enough to find themselves on the wrong end of her massive troll grade greatsword.</t>
+  </si>
+  <si>
+    <t>Freya Blackheart</t>
+  </si>
+  <si>
+    <t>The Great Cold</t>
   </si>
 </sst>
 </file>
@@ -799,10 +829,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4475C369-6A4F-4C74-96DE-3CDD122E599C}">
-  <dimension ref="A3:G54"/>
+  <dimension ref="A3:G60"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.85546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="14.28515625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="136.140625" style="1" customWidth="1"/>
@@ -1636,6 +1667,98 @@
         <v>119</v>
       </c>
     </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A57" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B57" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C57" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="D57" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E57" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="F57" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="G57" s="5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" ht="120" x14ac:dyDescent="0.25">
+      <c r="A58" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B58" t="s">
+        <v>121</v>
+      </c>
+      <c r="C58" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D58" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="E58" s="2">
+        <v>75</v>
+      </c>
+      <c r="F58" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G58" s="3" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" ht="135" x14ac:dyDescent="0.25">
+      <c r="A59" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="B59" t="s">
+        <v>123</v>
+      </c>
+      <c r="C59" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="D59" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="E59" s="2">
+        <v>85</v>
+      </c>
+      <c r="F59" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="G59" s="3" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" ht="120" x14ac:dyDescent="0.25">
+      <c r="A60" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="B60" t="s">
+        <v>129</v>
+      </c>
+      <c r="C60" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D60" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="E60" s="2">
+        <v>65</v>
+      </c>
+      <c r="F60" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G60" s="3" t="s">
+        <v>127</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
added lorebooks. more ui updates
</commit_message>
<xml_diff>
--- a/lores.xlsx
+++ b/lores.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\daeva\Desktop\Card_game\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0656AC25-0B0B-44FB-97CD-89A35F399ACB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7ED43EF-CD6E-4405-BAB5-56EB4C5FF719}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E9E6528D-FBE9-4018-A878-CDA73BAA7273}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E9E6528D-FBE9-4018-A878-CDA73BAA7273}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -285,9 +285,6 @@
     <t>Lightfoot Thunder</t>
   </si>
   <si>
-    <t>Eamon is a thirty nine year old Air Scout whose sharp wit and easygoing sarcasm make him a memorable, if somewhat unreliable, presence in the local taverns. Earning the nickname Lightfoot Thunder for his swift melee strikes and evasive maneuvers, he deliberately avoids the escalating war against the demon king by exclusively traveling between small villages to accept only the safest, lowest grade quests. This cautious approach ensures his coin purse stays reasonably full while completely eliminating the risk of facing actual danger, a lifestyle that suits his pragmatic mindset perfectly. His comfortable routine was entirely upended following a coincidental reunion with his longtime friend Alden, who guilted the reluctant scout into joining a far more dangerous expedition. While Eamon constantly complains about the sudden increase in peril, he has found a compelling reason to stick around. He has taken a keen interest in Alden’s young niece, secretly desiring a much closer and intimate relationship with her, even if his charming advances are currently falling flat.</t>
-  </si>
-  <si>
     <t>Yvaine Ashcroft</t>
   </si>
   <si>
@@ -424,6 +421,9 @@
   </si>
   <si>
     <t>The Great Cold</t>
+  </si>
+  <si>
+    <t>Eamon is a thirty nine year old Air Scout whose sharp wit and easygoing sarcasm make him a memorable, if somewhat unreliable, presence in the local taverns. Earning the nickname Lightfoot Thunder for his swift melee strikes and evasive maneuvers, he deliberately avoids the escalating war against the demon king by exclusively traveling between small villages to accept only the safest, lowest grade quests. This cautious approach ensures his coin purse stays reasonably full while completely eliminating the risk of facing actual danger, a lifestyle that suits his pragmatic mindset perfectly. His comfortable routine was entirely upended following a coincidental reunion with his longtime friend Alden, who guilted the reluctant scout into joining a far more dangerous expedition. While Eamon constantly complains about the sudden increase in peril, he has found a compelling reason to stick around. He has taken a keen interest in Alden’s young niece, secretly desiring to impress her, even if his charming advances are currently falling flat.</t>
   </si>
 </sst>
 </file>
@@ -1365,15 +1365,15 @@
         <v>8</v>
       </c>
       <c r="G35" s="3" t="s">
-        <v>83</v>
+        <v>129</v>
       </c>
     </row>
     <row r="36" spans="1:7" ht="120" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B36" s="2" t="s">
         <v>84</v>
-      </c>
-      <c r="B36" s="2" t="s">
-        <v>85</v>
       </c>
       <c r="C36" s="2" t="s">
         <v>55</v>
@@ -1388,7 +1388,7 @@
         <v>15</v>
       </c>
       <c r="G36" s="3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
@@ -1416,10 +1416,10 @@
     </row>
     <row r="40" spans="1:7" ht="120" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="B40" t="s">
         <v>87</v>
-      </c>
-      <c r="B40" t="s">
-        <v>88</v>
       </c>
       <c r="C40" s="2" t="s">
         <v>51</v>
@@ -1434,15 +1434,15 @@
         <v>43</v>
       </c>
       <c r="G40" s="3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="41" spans="1:7" ht="120" x14ac:dyDescent="0.25">
       <c r="A41" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="B41" t="s">
         <v>90</v>
-      </c>
-      <c r="B41" t="s">
-        <v>91</v>
       </c>
       <c r="C41" s="2" t="s">
         <v>6</v>
@@ -1457,15 +1457,15 @@
         <v>8</v>
       </c>
       <c r="G41" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="42" spans="1:7" ht="120" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B42" s="2" t="s">
         <v>93</v>
-      </c>
-      <c r="B42" s="2" t="s">
-        <v>94</v>
       </c>
       <c r="C42" s="2" t="s">
         <v>55</v>
@@ -1480,7 +1480,7 @@
         <v>8</v>
       </c>
       <c r="G42" s="3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
@@ -1508,10 +1508,10 @@
     </row>
     <row r="46" spans="1:7" ht="135" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B46" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C46" s="2" t="s">
         <v>51</v>
@@ -1526,18 +1526,18 @@
         <v>8</v>
       </c>
       <c r="G46" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="47" spans="1:7" ht="150" x14ac:dyDescent="0.25">
       <c r="A47" s="6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B47" t="s">
+        <v>100</v>
+      </c>
+      <c r="C47" s="2" t="s">
         <v>101</v>
-      </c>
-      <c r="C47" s="2" t="s">
-        <v>102</v>
       </c>
       <c r="D47" s="2" t="s">
         <v>33</v>
@@ -1549,21 +1549,21 @@
         <v>8</v>
       </c>
       <c r="G47" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="48" spans="1:7" ht="135" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B48" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C48" s="2" t="s">
         <v>13</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E48" s="2">
         <v>45</v>
@@ -1572,7 +1572,7 @@
         <v>43</v>
       </c>
       <c r="G48" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
@@ -1600,16 +1600,16 @@
     </row>
     <row r="52" spans="1:7" ht="150" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B52" t="s">
+        <v>109</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="D52" s="2" t="s">
         <v>110</v>
-      </c>
-      <c r="C52" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="D52" s="2" t="s">
-        <v>111</v>
       </c>
       <c r="E52" s="2">
         <v>90</v>
@@ -1618,21 +1618,21 @@
         <v>8</v>
       </c>
       <c r="G52" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="53" spans="1:7" ht="135" x14ac:dyDescent="0.25">
       <c r="A53" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B53" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C53" s="2" t="s">
         <v>61</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E53" s="2">
         <v>100</v>
@@ -1641,30 +1641,30 @@
         <v>8</v>
       </c>
       <c r="G53" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="54" spans="1:7" ht="150" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B54" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C54" s="2" t="s">
         <v>51</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E54" s="2">
         <v>95</v>
       </c>
       <c r="F54" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="G54" s="3" t="s">
         <v>118</v>
-      </c>
-      <c r="G54" s="3" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
@@ -1692,10 +1692,10 @@
     </row>
     <row r="58" spans="1:7" ht="120" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B58" t="s">
         <v>120</v>
-      </c>
-      <c r="B58" t="s">
-        <v>121</v>
       </c>
       <c r="C58" s="2" t="s">
         <v>42</v>
@@ -1704,24 +1704,24 @@
         <v>72</v>
       </c>
       <c r="E58" s="2">
-        <v>75</v>
+        <v>60</v>
       </c>
       <c r="F58" s="2" t="s">
         <v>8</v>
       </c>
       <c r="G58" s="3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="59" spans="1:7" ht="135" x14ac:dyDescent="0.25">
       <c r="A59" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="B59" t="s">
         <v>122</v>
       </c>
-      <c r="B59" t="s">
+      <c r="C59" s="2" t="s">
         <v>123</v>
-      </c>
-      <c r="C59" s="2" t="s">
-        <v>124</v>
       </c>
       <c r="D59" s="2" t="s">
         <v>72</v>
@@ -1730,18 +1730,18 @@
         <v>85</v>
       </c>
       <c r="F59" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="G59" s="3" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="60" spans="1:7" ht="120" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="B60" t="s">
         <v>128</v>
-      </c>
-      <c r="B60" t="s">
-        <v>129</v>
       </c>
       <c r="C60" s="2" t="s">
         <v>51</v>
@@ -1756,7 +1756,7 @@
         <v>8</v>
       </c>
       <c r="G60" s="3" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
   </sheetData>

</xml_diff>